<commit_message>
PU_projekt.xlsx: Utvecklingskostnad/Anskaffning bekräftade mot fysiskt kort
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/PU_projekt.xlsx
+++ b/kortdata/PU_projekt.xlsx
@@ -12,7 +12,6 @@
     <sheet name="Produktion" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="Kolumner" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="Källa och kontroll" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Frågor" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -512,7 +511,7 @@
       </c>
       <c r="G1" s="1" t="inlineStr">
         <is>
-          <t>Kostnad (Mkr)</t>
+          <t>Utvecklingskostnad (Mkr)</t>
         </is>
       </c>
       <c r="H1" s="1" t="inlineStr">
@@ -8006,7 +8005,7 @@
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>Anskaffning · Utvecklingskostnad · BTA · H · Q</t>
+          <t>H · Q · BTA · Utvecklingskostnad · Anskaffning</t>
         </is>
       </c>
     </row>
@@ -8040,7 +8039,7 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>Passera nämnden · Riskbuffert · Hållbarhetskrav · Kvalitetskrav · Tidspåverkan</t>
+          <t>BTA · Utvecklingskostnad · Anskaffning · Riskbuffert · Passera nämnden · Hållbarhetskrav · Kvalitetskrav · Tidspåverkan</t>
         </is>
       </c>
     </row>
@@ -11446,7 +11445,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Kostnad (Mkr)</t>
+          <t>Utvecklingskostnad (Mkr)</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
@@ -11461,7 +11460,7 @@
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Tryckt under etiketten 'Anskaffning' — se Frågor</t>
+          <t>Kostnad för att ta projektet i Skede 1</t>
         </is>
       </c>
     </row>
@@ -11481,11 +11480,7 @@
           <t>Ja</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>Tryckt under etiketten 'Utvecklingskostnad' — se Frågor</t>
-        </is>
-      </c>
+      <c r="D9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -12212,7 +12207,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B10"/>
+  <dimension ref="A1:B11"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -12330,54 +12325,24 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>Etiketter</t>
+        </is>
+      </c>
+      <c r="B10" t="inlineStr">
+        <is>
+          <t>Bekräftat mot fysiskt kort (BRF Eldningen): Utvecklingskostnad = CSV 'Kostnad', Anskaffning = CSV 'Anskaffning'. Textordningen i PDF:en följer inte layouten.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>Byggd med</t>
         </is>
       </c>
-      <c r="B10" t="inlineStr">
+      <c r="B11" t="inlineStr">
         <is>
           <t>verktyg/bygg_pu_projekt_excel.py</t>
-        </is>
-      </c>
-    </row>
-  </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-</worksheet>
-</file>
-
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <sheetPr>
-    <outlinePr summaryBelow="1" summaryRight="1"/>
-    <pageSetUpPr/>
-  </sheetPr>
-  <dimension ref="A1:B2"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
-  <cols>
-    <col width="60" customWidth="1" min="1" max="1"/>
-    <col width="110" customWidth="1" min="2" max="2"/>
-  </cols>
-  <sheetData>
-    <row r="1">
-      <c r="A1" s="1" t="inlineStr">
-        <is>
-          <t>Fråga</t>
-        </is>
-      </c>
-      <c r="B1" s="1" t="inlineStr">
-        <is>
-          <t>Bakgrund</t>
-        </is>
-      </c>
-    </row>
-    <row r="2">
-      <c r="A2" s="2" t="inlineStr">
-        <is>
-          <t>Vilket värde står under 'Anskaffning' respektive 'Utvecklingskostnad' på framsidan?</t>
-        </is>
-      </c>
-      <c r="B2" s="2" t="inlineStr">
-        <is>
-          <t>Textordningen i tryckfilen är 'Anskaffning, Utvecklingskostnad, BTA, 2 Mkr, 33 Mkr'. CSV har Kostnad=2 och Anskaffning=33. Om etiketterna följer värdeordningen är Anskaffning=2 och Utvecklingskostnad=33 på kortet, dvs. CSV-namnen är omvända. Behöver bekräftas mot ett fysiskt kort.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Skede 1 (Projektutveckling) i motorn; Förvaltningen startar från dess utfall
- motor/pu.py: tryckta PU-brädet, PC-val, startprojekt, projektbank, händelsekort (vanliga + special),
  hörn, nämnd 4.1, komplettering 4.2, placering 4.3 (kapacitet), kvartertyp 4.4, ABT 5.1.
- motor/pu_strategi.py: fyra bottar (balanserad, försiktig, expansiv, bostad).
- PU_projekt.xlsx: brickornas former (Antal rutor, Form) och omtryck Regnbågen BTA 1750.
- Regelboken: Stadsbyggnadskontoret vid start/passering, Skönhetsrådet ökar kraven (som brädet),
  tomtkostnad 10 Mkr, BYA = fotavtryck.
- tester/test_pu.py.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/PU_projekt.xlsx
+++ b/kortdata/PU_projekt.xlsx
@@ -432,7 +432,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:AT46"/>
+  <dimension ref="A1:AV46"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -481,6 +481,8 @@
     <col width="14" customWidth="1" min="44" max="44"/>
     <col width="14" customWidth="1" min="45" max="45"/>
     <col width="14" customWidth="1" min="46" max="46"/>
+    <col width="14" customWidth="1" min="47" max="47"/>
+    <col width="14" customWidth="1" min="48" max="48"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -641,75 +643,85 @@
       </c>
       <c r="AF1" s="1" t="inlineStr">
         <is>
+          <t>Antal rutor</t>
+        </is>
+      </c>
+      <c r="AG1" s="1" t="inlineStr">
+        <is>
+          <t>Form (rutor)</t>
+        </is>
+      </c>
+      <c r="AH1" s="1" t="inlineStr">
+        <is>
           <t>Förekomst</t>
         </is>
       </c>
-      <c r="AG1" s="1" t="inlineStr">
+      <c r="AI1" s="1" t="inlineStr">
         <is>
           <t>Formfaktor</t>
         </is>
       </c>
-      <c r="AH1" s="1" t="inlineStr">
+      <c r="AJ1" s="1" t="inlineStr">
         <is>
           <t>Linjetyp</t>
         </is>
       </c>
-      <c r="AI1" s="1" t="inlineStr">
+      <c r="AK1" s="1" t="inlineStr">
         <is>
           <t>Antal krav</t>
         </is>
       </c>
-      <c r="AJ1" s="1" t="inlineStr">
+      <c r="AL1" s="1" t="inlineStr">
         <is>
           <t>STA</t>
         </is>
       </c>
-      <c r="AK1" s="1" t="inlineStr">
+      <c r="AM1" s="1" t="inlineStr">
         <is>
           <t>KOM</t>
         </is>
       </c>
-      <c r="AL1" s="1" t="inlineStr">
+      <c r="AN1" s="1" t="inlineStr">
         <is>
           <t>SAM</t>
         </is>
       </c>
-      <c r="AM1" s="1" t="inlineStr">
+      <c r="AO1" s="1" t="inlineStr">
         <is>
           <t>NOG</t>
         </is>
       </c>
-      <c r="AN1" s="1" t="inlineStr">
+      <c r="AP1" s="1" t="inlineStr">
         <is>
           <t>INN</t>
         </is>
       </c>
-      <c r="AO1" s="1" t="inlineStr">
+      <c r="AQ1" s="1" t="inlineStr">
         <is>
           <t>ABM</t>
         </is>
       </c>
-      <c r="AP1" s="1" t="inlineStr">
+      <c r="AR1" s="1" t="inlineStr">
         <is>
           <t>Skalfaktor</t>
         </is>
       </c>
-      <c r="AQ1" s="1" t="inlineStr">
+      <c r="AS1" s="1" t="inlineStr">
         <is>
           <t>Intäkt/kvm nu</t>
         </is>
       </c>
-      <c r="AR1" s="1" t="inlineStr">
+      <c r="AT1" s="1" t="inlineStr">
         <is>
           <t>Förslag intäkt</t>
         </is>
       </c>
-      <c r="AS1" s="1" t="inlineStr">
+      <c r="AU1" s="1" t="inlineStr">
         <is>
           <t>Bildprompt (en)</t>
         </is>
       </c>
-      <c r="AT1" s="1" t="inlineStr">
+      <c r="AV1" s="1" t="inlineStr">
         <is>
           <t>Antal exemplar</t>
         </is>
@@ -832,32 +844,32 @@
         </is>
       </c>
       <c r="AF2" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG2" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [1, 2]]</t>
+        </is>
+      </c>
+      <c r="AH2" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG2" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH2" s="2" t="inlineStr">
+      <c r="AI2" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ2" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI2" s="2" t="inlineStr"/>
-      <c r="AJ2" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK2" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AK2" s="2" t="inlineStr"/>
       <c r="AL2" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="AM2" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN2" s="2" t="inlineStr">
         <is>
@@ -867,19 +879,27 @@
       <c r="AO2" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP2" s="2" t="inlineStr"/>
+      <c r="AP2" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ2" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR2" s="2" t="inlineStr"/>
+      <c r="AS2" s="2" t="n">
         <v>43</v>
       </c>
-      <c r="AR2" s="2" t="n">
+      <c r="AT2" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS2" s="2" t="inlineStr">
+      <c r="AU2" s="2" t="inlineStr">
         <is>
           <t>fire, burning flames, ember glow</t>
         </is>
       </c>
-      <c r="AT2" s="2" t="n">
+      <c r="AV2" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1000,54 +1020,62 @@
         </is>
       </c>
       <c r="AF3" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG3" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 0], [2, 1], [3, 1]]</t>
+        </is>
+      </c>
+      <c r="AH3" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH3" s="2" t="inlineStr">
+      <c r="AI3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ3" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI3" s="2" t="inlineStr"/>
-      <c r="AJ3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK3" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN3" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO3" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP3" s="2" t="inlineStr"/>
+      <c r="AK3" s="2" t="inlineStr"/>
+      <c r="AL3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM3" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP3" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ3" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR3" s="2" t="inlineStr"/>
+      <c r="AS3" s="2" t="n">
         <v>40.66666667</v>
       </c>
-      <c r="AR3" s="2" t="n">
+      <c r="AT3" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS3" s="2" t="inlineStr">
+      <c r="AU3" s="2" t="inlineStr">
         <is>
           <t>forest glade, clearing, sunlight through trees</t>
         </is>
       </c>
-      <c r="AT3" s="2" t="n">
+      <c r="AV3" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1168,32 +1196,32 @@
         </is>
       </c>
       <c r="AF4" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AG4" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [2, 0], [2, 1], [3, 0], [3, 1]]</t>
+        </is>
+      </c>
+      <c r="AH4" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG4" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH4" s="2" t="inlineStr">
+      <c r="AI4" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ4" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI4" s="2" t="inlineStr"/>
-      <c r="AJ4" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK4" s="2" t="n">
-        <v>2</v>
-      </c>
+      <c r="AK4" s="2" t="inlineStr"/>
       <c r="AL4" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
       <c r="AM4" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN4" s="2" t="inlineStr">
         <is>
@@ -1203,19 +1231,27 @@
       <c r="AO4" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP4" s="2" t="inlineStr"/>
+      <c r="AP4" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ4" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR4" s="2" t="inlineStr"/>
+      <c r="AS4" s="2" t="n">
         <v>39.5</v>
       </c>
-      <c r="AR4" s="2" t="n">
+      <c r="AT4" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS4" s="2" t="inlineStr">
+      <c r="AU4" s="2" t="inlineStr">
         <is>
           <t>wide horizon, distant skyline, open sky</t>
         </is>
       </c>
-      <c r="AT4" s="2" t="n">
+      <c r="AV4" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1336,54 +1372,62 @@
         </is>
       </c>
       <c r="AF5" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG5" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG5" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [2, 0], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH5" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI5" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AH5" s="2" t="inlineStr">
+      <c r="AJ5" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI5" s="2" t="n">
+      <c r="AK5" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK5" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL5" s="2" t="n">
-        <v>1</v>
+      <c r="AL5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN5" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN5" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO5" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP5" s="2" t="inlineStr"/>
+      <c r="AP5" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ5" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR5" s="2" t="inlineStr"/>
+      <c r="AS5" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="AR5" s="2" t="n">
+      <c r="AT5" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="AS5" s="2" t="inlineStr">
+      <c r="AU5" s="2" t="inlineStr">
         <is>
           <t>rocky cliff, stone crag, rugged outcrop</t>
         </is>
       </c>
-      <c r="AT5" s="2" t="n">
+      <c r="AV5" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1502,56 +1546,64 @@
         </is>
       </c>
       <c r="AF6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG6" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG6" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [2, 0], [3, 0], [4, 0], [4, 1]]</t>
+        </is>
+      </c>
+      <c r="AH6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI6" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AH6" s="2" t="inlineStr">
+      <c r="AJ6" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI6" s="2" t="n">
+      <c r="AK6" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AJ6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK6" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL6" s="2" t="n">
-        <v>1</v>
+      <c r="AL6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM6" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO6" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP6" s="2" t="inlineStr"/>
-      <c r="AQ6" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO6" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ6" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR6" s="2" t="inlineStr"/>
+      <c r="AS6" s="2" t="n">
         <v>53.14285714</v>
       </c>
-      <c r="AR6" s="2" t="n">
+      <c r="AT6" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="AS6" s="2" t="inlineStr">
+      <c r="AU6" s="2" t="inlineStr">
         <is>
           <t>golden grain, wheat sheaf, harvest field</t>
         </is>
       </c>
-      <c r="AT6" s="2" t="n">
+      <c r="AV6" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1672,56 +1724,64 @@
         </is>
       </c>
       <c r="AF7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG7" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG7" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 0], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH7" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI7" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AH7" s="2" t="inlineStr">
+      <c r="AJ7" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI7" s="2" t="n">
+      <c r="AK7" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AJ7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK7" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM7" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AL7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM7" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AN7" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AO7" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP7" s="2" t="inlineStr"/>
+      <c r="AO7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP7" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ7" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR7" s="2" t="inlineStr"/>
+      <c r="AS7" s="2" t="n">
         <v>52.8</v>
       </c>
-      <c r="AR7" s="2" t="n">
+      <c r="AT7" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="AS7" s="2" t="inlineStr">
+      <c r="AU7" s="2" t="inlineStr">
         <is>
           <t>sunflower, golden petals, summer bloom</t>
         </is>
       </c>
-      <c r="AT7" s="2" t="n">
+      <c r="AV7" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -1842,26 +1902,26 @@
         </is>
       </c>
       <c r="AF8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG8" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AH8" s="2" t="inlineStr">
+      <c r="AG8" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 1], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI8" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AJ8" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ8" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AK8" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL8" s="2" t="inlineStr">
         <is>
@@ -1869,7 +1929,7 @@
         </is>
       </c>
       <c r="AM8" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AN8" s="2" t="inlineStr">
         <is>
@@ -1877,21 +1937,29 @@
         </is>
       </c>
       <c r="AO8" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP8" s="2" t="inlineStr"/>
+        <v>2</v>
+      </c>
+      <c r="AP8" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ8" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR8" s="2" t="inlineStr"/>
+      <c r="AS8" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="AR8" s="2" t="n">
+      <c r="AT8" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="AS8" s="2" t="inlineStr">
+      <c r="AU8" s="2" t="inlineStr">
         <is>
           <t>reflection, mirror lake, still water</t>
         </is>
       </c>
-      <c r="AT8" s="2" t="n">
+      <c r="AV8" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2012,56 +2080,64 @@
         </is>
       </c>
       <c r="AF9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG9" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH9" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="AG9" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [0, 2]]</t>
+        </is>
+      </c>
+      <c r="AH9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ9" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI9" s="2" t="n">
+      <c r="AK9" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL9" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN9" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO9" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP9" s="2" t="inlineStr"/>
+      <c r="AL9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN9" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP9" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ9" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR9" s="2" t="inlineStr"/>
+      <c r="AS9" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="AR9" s="2" t="n">
+      <c r="AT9" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="AS9" s="2" t="inlineStr">
+      <c r="AU9" s="2" t="inlineStr">
         <is>
           <t>forest path, winding trail, woodland walk</t>
         </is>
       </c>
-      <c r="AT9" s="2" t="n">
+      <c r="AV9" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2180,32 +2256,32 @@
         </is>
       </c>
       <c r="AF10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG10" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AH10" s="2" t="inlineStr">
+      <c r="AG10" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [0, 2], [0, 3], [1, 2], [1, 3], [2, 3], [3, 3]]</t>
+        </is>
+      </c>
+      <c r="AH10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI10" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ10" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI10" s="2" t="n">
+      <c r="AK10" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AJ10" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK10" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL10" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AL10" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AM10" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AN10" s="2" t="inlineStr">
         <is>
@@ -2215,19 +2291,27 @@
       <c r="AO10" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP10" s="2" t="inlineStr"/>
+      <c r="AP10" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
       <c r="AQ10" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR10" s="2" t="inlineStr"/>
+      <c r="AS10" s="2" t="n">
         <v>59.5</v>
       </c>
-      <c r="AR10" s="2" t="n">
+      <c r="AT10" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="AS10" s="2" t="inlineStr">
+      <c r="AU10" s="2" t="inlineStr">
         <is>
           <t>stone vault, arched ceiling, ancient architecture</t>
         </is>
       </c>
-      <c r="AT10" s="2" t="n">
+      <c r="AV10" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2356,56 +2440,64 @@
         </is>
       </c>
       <c r="AF11" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG11" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [0, 2], [1, 1]]</t>
+        </is>
+      </c>
+      <c r="AH11" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG11" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH11" s="2" t="inlineStr">
+      <c r="AI11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ11" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI11" s="2" t="inlineStr"/>
-      <c r="AJ11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK11" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM11" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AK11" s="2" t="inlineStr"/>
+      <c r="AL11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM11" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AN11" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AO11" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP11" s="2" t="n">
-        <v>1</v>
+      <c r="AO11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP11" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ11" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR11" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS11" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AR11" s="2" t="n">
+      <c r="AT11" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS11" s="2" t="inlineStr">
+      <c r="AU11" s="2" t="inlineStr">
         <is>
           <t>dragon lair, cave, mythical den</t>
         </is>
       </c>
-      <c r="AT11" s="2" t="n">
+      <c r="AV11" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2534,56 +2626,64 @@
         </is>
       </c>
       <c r="AF12" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG12" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [0, 2], [1, 0], [1, 1], [1, 2]]</t>
+        </is>
+      </c>
+      <c r="AH12" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG12" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH12" s="2" t="inlineStr">
+      <c r="AI12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ12" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI12" s="2" t="inlineStr"/>
-      <c r="AJ12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK12" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM12" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AK12" s="2" t="inlineStr"/>
+      <c r="AL12" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM12" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AN12" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AO12" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP12" s="2" t="n">
+      <c r="AO12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP12" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ12" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR12" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ12" s="2" t="n">
+      <c r="AS12" s="2" t="n">
         <v>42</v>
       </c>
-      <c r="AR12" s="2" t="n">
+      <c r="AT12" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS12" s="2" t="inlineStr">
+      <c r="AU12" s="2" t="inlineStr">
         <is>
           <t>somersault, tumble, playful roll</t>
         </is>
       </c>
-      <c r="AT12" s="2" t="n">
+      <c r="AV12" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2718,23 +2818,23 @@
       <c r="AF13" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH13" s="2" t="inlineStr">
+      <c r="AG13" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 1], [1, 0], [1, 1]]</t>
+        </is>
+      </c>
+      <c r="AH13" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ13" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI13" s="2" t="inlineStr"/>
-      <c r="AJ13" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK13" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AK13" s="2" t="inlineStr"/>
       <c r="AL13" s="2" t="inlineStr">
         <is>
           <t>-</t>
@@ -2749,23 +2849,31 @@
         </is>
       </c>
       <c r="AO13" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP13" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP13" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ13" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR13" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ13" s="2" t="n">
+      <c r="AS13" s="2" t="n">
         <v>45.33333333</v>
       </c>
-      <c r="AR13" s="2" t="n">
+      <c r="AT13" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS13" s="2" t="inlineStr">
+      <c r="AU13" s="2" t="inlineStr">
         <is>
           <t>ladybug, spotted beetle, garden friend</t>
         </is>
       </c>
-      <c r="AT13" s="2" t="n">
+      <c r="AV13" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2794,7 +2902,7 @@
         </is>
       </c>
       <c r="F14" s="2" t="n">
-        <v>2000</v>
+        <v>1750</v>
       </c>
       <c r="G14" s="2" t="n">
         <v>7</v>
@@ -2890,56 +2998,64 @@
         </is>
       </c>
       <c r="AF14" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG14" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG14" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [2, 0], [2, 1], [3, 0], [4, 0]]</t>
+        </is>
+      </c>
+      <c r="AH14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI14" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="AH14" s="2" t="inlineStr">
+      <c r="AJ14" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI14" s="2" t="n">
+      <c r="AK14" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AJ14" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK14" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL14" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AM14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN14" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO14" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP14" s="2" t="n">
-        <v>1</v>
+      <c r="AM14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP14" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ14" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR14" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS14" s="2" t="n">
         <v>57.5</v>
       </c>
-      <c r="AR14" s="2" t="n">
+      <c r="AT14" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="AS14" s="2" t="inlineStr">
+      <c r="AU14" s="2" t="inlineStr">
         <is>
           <t>rainbow, colorful arc, after rain</t>
         </is>
       </c>
-      <c r="AT14" s="2" t="n">
+      <c r="AV14" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3066,29 +3182,29 @@
         </is>
       </c>
       <c r="AF15" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG15" s="2" t="n">
-        <v>3</v>
-      </c>
-      <c r="AH15" s="2" t="inlineStr">
-        <is>
-          <t>prickad</t>
-        </is>
+        <v>5</v>
+      </c>
+      <c r="AG15" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 0], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH15" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AI15" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ15" s="2" t="n">
-        <v>1</v>
+      <c r="AJ15" s="2" t="inlineStr">
+        <is>
+          <t>prickad</t>
+        </is>
       </c>
       <c r="AK15" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL15" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>3</v>
+      </c>
+      <c r="AL15" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AM15" s="2" t="n">
         <v>1</v>
@@ -3101,21 +3217,29 @@
       <c r="AO15" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP15" s="2" t="n">
-        <v>1</v>
+      <c r="AP15" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR15" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS15" s="2" t="n">
         <v>50.4</v>
       </c>
-      <c r="AR15" s="2" t="n">
+      <c r="AT15" s="2" t="n">
         <v>53</v>
       </c>
-      <c r="AS15" s="2" t="inlineStr">
+      <c r="AU15" s="2" t="inlineStr">
         <is>
           <t>treasure chest, golden chest, pirate loot</t>
         </is>
       </c>
-      <c r="AT15" s="2" t="n">
+      <c r="AV15" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3240,56 +3364,64 @@
         </is>
       </c>
       <c r="AF16" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG16" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG16" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [2, 0], [3, 0], [4, 0]]</t>
+        </is>
+      </c>
+      <c r="AH16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI16" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AH16" s="2" t="inlineStr">
+      <c r="AJ16" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI16" s="2" t="n">
+      <c r="AK16" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AJ16" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK16" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL16" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AM16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN16" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO16" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP16" s="2" t="n">
-        <v>1</v>
+      <c r="AM16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP16" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ16" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR16" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS16" s="2" t="n">
         <v>54.28571429</v>
       </c>
-      <c r="AR16" s="2" t="n">
+      <c r="AT16" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="AS16" s="2" t="inlineStr">
+      <c r="AU16" s="2" t="inlineStr">
         <is>
           <t>wild strawberry patch, secret spot, hidden paradise</t>
         </is>
       </c>
-      <c r="AT16" s="2" t="n">
+      <c r="AV16" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3416,58 +3548,66 @@
         </is>
       </c>
       <c r="AF17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG17" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AH17" s="2" t="inlineStr">
+      <c r="AG17" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 0]]</t>
+        </is>
+      </c>
+      <c r="AH17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI17" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AJ17" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ17" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AK17" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AL17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AM17" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AL17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM17" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AN17" s="2" t="inlineStr">
         <is>
           <t>-</t>
         </is>
       </c>
-      <c r="AO17" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP17" s="2" t="n">
+      <c r="AO17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP17" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ17" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR17" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ17" s="2" t="n">
+      <c r="AS17" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="AR17" s="2" t="n">
+      <c r="AT17" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="AS17" s="2" t="inlineStr">
+      <c r="AU17" s="2" t="inlineStr">
         <is>
           <t>star seed, cosmic sprout, celestial growth</t>
         </is>
       </c>
-      <c r="AT17" s="2" t="n">
+      <c r="AV17" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3592,56 +3732,64 @@
         </is>
       </c>
       <c r="AF18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG18" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AH18" s="2" t="inlineStr">
+      <c r="AG18" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 1], [1, 1], [2, 0], [2, 1], [3, 1]]</t>
+        </is>
+      </c>
+      <c r="AH18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI18" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AJ18" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI18" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AK18" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL18" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AL18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN18" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN18" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO18" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP18" s="2" t="n">
+      <c r="AP18" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ18" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR18" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ18" s="2" t="n">
+      <c r="AS18" s="2" t="n">
         <v>53.6</v>
       </c>
-      <c r="AR18" s="2" t="n">
+      <c r="AT18" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="AS18" s="2" t="inlineStr">
+      <c r="AU18" s="2" t="inlineStr">
         <is>
           <t>enchanted forest, magical woods, fairy tale grove</t>
         </is>
       </c>
-      <c r="AT18" s="2" t="n">
+      <c r="AV18" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3766,29 +3914,29 @@
         </is>
       </c>
       <c r="AF19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG19" s="2" t="n">
         <v>6</v>
       </c>
-      <c r="AH19" s="2" t="inlineStr">
+      <c r="AG19" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 1], [0, 3], [1, 0], [1, 1], [1, 2], [1, 3]]</t>
+        </is>
+      </c>
+      <c r="AH19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI19" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AJ19" s="2" t="inlineStr">
         <is>
           <t>prickad</t>
         </is>
       </c>
-      <c r="AI19" s="2" t="n">
+      <c r="AK19" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK19" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL19" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AL19" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AM19" s="2" t="n">
         <v>1</v>
@@ -3799,23 +3947,31 @@
         </is>
       </c>
       <c r="AO19" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AP19" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP19" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ19" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AR19" s="2" t="n">
         <v>1.05</v>
       </c>
-      <c r="AQ19" s="2" t="n">
+      <c r="AS19" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="AR19" s="2" t="n">
+      <c r="AT19" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="AS19" s="2" t="inlineStr">
+      <c r="AU19" s="2" t="inlineStr">
         <is>
           <t>coltsfoot flower, early spring bloom, yellow wildflower</t>
         </is>
       </c>
-      <c r="AT19" s="2" t="n">
+      <c r="AV19" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3946,52 +4102,60 @@
       <c r="AF20" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG20" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH20" s="2" t="inlineStr">
+      <c r="AG20" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 1]]</t>
+        </is>
+      </c>
+      <c r="AH20" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ20" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI20" s="2" t="inlineStr"/>
-      <c r="AJ20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK20" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AK20" s="2" t="inlineStr"/>
       <c r="AL20" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM20" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO20" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP20" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AQ20" s="2" t="n">
+      <c r="AN20" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ20" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR20" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS20" s="2" t="n">
         <v>46.66666667</v>
       </c>
-      <c r="AR20" s="2" t="n">
+      <c r="AT20" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="AS20" s="2" t="inlineStr">
+      <c r="AU20" s="2" t="inlineStr">
         <is>
           <t>the pawn, chess piece, opening move</t>
         </is>
       </c>
-      <c r="AT20" s="2" t="n">
+      <c r="AV20" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4120,54 +4284,62 @@
         </is>
       </c>
       <c r="AF21" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG21" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 1], [2, 0], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH21" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG21" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH21" s="2" t="inlineStr">
+      <c r="AI21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ21" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI21" s="2" t="inlineStr"/>
-      <c r="AJ21" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK21" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AK21" s="2" t="inlineStr"/>
       <c r="AL21" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM21" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO21" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP21" s="2" t="n">
+      <c r="AN21" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO21" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ21" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR21" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ21" s="2" t="n">
+      <c r="AS21" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AR21" s="2" t="n">
+      <c r="AT21" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="AS21" s="2" t="inlineStr">
+      <c r="AU21" s="2" t="inlineStr">
         <is>
           <t>the queen, chess piece, powerful move</t>
         </is>
       </c>
-      <c r="AT21" s="2" t="n">
+      <c r="AV21" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4296,54 +4468,62 @@
         </is>
       </c>
       <c r="AF22" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG22" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [2, 0], [2, 1], [2, 2]]</t>
+        </is>
+      </c>
+      <c r="AH22" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG22" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH22" s="2" t="inlineStr">
+      <c r="AI22" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ22" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI22" s="2" t="inlineStr"/>
-      <c r="AJ22" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK22" s="2" t="n">
-        <v>1</v>
-      </c>
+      <c r="AK22" s="2" t="inlineStr"/>
       <c r="AL22" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AM22" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO22" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP22" s="2" t="n">
+      <c r="AN22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO22" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ22" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR22" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ22" s="2" t="n">
+      <c r="AS22" s="2" t="n">
         <v>41.71428571</v>
       </c>
-      <c r="AR22" s="2" t="n">
+      <c r="AT22" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="AS22" s="2" t="inlineStr">
+      <c r="AU22" s="2" t="inlineStr">
         <is>
           <t>the gambit, chess sacrifice, strategic opening</t>
         </is>
       </c>
-      <c r="AT22" s="2" t="n">
+      <c r="AV22" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4470,56 +4650,64 @@
         </is>
       </c>
       <c r="AF23" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG23" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG23" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 0], [2, 1], [3, 0], [4, 0]]</t>
+        </is>
+      </c>
+      <c r="AH23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI23" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AH23" s="2" t="inlineStr">
+      <c r="AJ23" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI23" s="2" t="n">
+      <c r="AK23" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK23" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL23" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN23" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO23" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP23" s="2" t="n">
-        <v>1</v>
+        <v>1</v>
+      </c>
+      <c r="AM23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN23" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP23" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR23" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS23" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="AR23" s="2" t="n">
+      <c r="AT23" s="2" t="n">
         <v>55</v>
       </c>
-      <c r="AS23" s="2" t="inlineStr">
+      <c r="AU23" s="2" t="inlineStr">
         <is>
           <t>the king, chess piece, royal protection</t>
         </is>
       </c>
-      <c r="AT23" s="2" t="n">
+      <c r="AV23" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4648,56 +4836,64 @@
         </is>
       </c>
       <c r="AF24" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG24" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG24" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 0], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI24" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AH24" s="2" t="inlineStr">
+      <c r="AJ24" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI24" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ24" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AK24" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL24" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM24" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO24" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP24" s="2" t="n">
+      <c r="AN24" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO24" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ24" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR24" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ24" s="2" t="n">
+      <c r="AS24" s="2" t="n">
         <v>48.8</v>
       </c>
-      <c r="AR24" s="2" t="n">
+      <c r="AT24" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="AS24" s="2" t="inlineStr">
+      <c r="AU24" s="2" t="inlineStr">
         <is>
           <t>the bishop, chess piece, diagonal move</t>
         </is>
       </c>
-      <c r="AT24" s="2" t="n">
+      <c r="AV24" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -4826,58 +5022,66 @@
         </is>
       </c>
       <c r="AF25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH25" s="2" t="inlineStr">
+        <v>4</v>
+      </c>
+      <c r="AG25" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ25" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI25" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ25" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AK25" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL25" s="2" t="n">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="AL25" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM25" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN25" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO25" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP25" s="2" t="n">
+      <c r="AN25" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO25" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP25" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ25" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR25" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ25" s="2" t="n">
+      <c r="AS25" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="AR25" s="2" t="n">
+      <c r="AT25" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="AS25" s="2" t="inlineStr">
+      <c r="AU25" s="2" t="inlineStr">
         <is>
           <t>the countermove, chess response, defensive play</t>
         </is>
       </c>
-      <c r="AT25" s="2" t="n">
+      <c r="AV25" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5006,22 +5210,24 @@
         </is>
       </c>
       <c r="AF26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH26" s="2" t="inlineStr">
+        <v>2</v>
+      </c>
+      <c r="AG26" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0]]</t>
+        </is>
+      </c>
+      <c r="AH26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ26" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI26" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ26" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AK26" s="2" t="n">
         <v>1</v>
       </c>
@@ -5031,29 +5237,35 @@
       <c r="AM26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN26" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN26" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO26" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP26" s="2" t="n">
-        <v>1</v>
+      <c r="AP26" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR26" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS26" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="AR26" s="2" t="n">
+      <c r="AT26" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="AS26" s="2" t="inlineStr">
+      <c r="AU26" s="2" t="inlineStr">
         <is>
           <t>castling, chess maneuver, king safety</t>
         </is>
       </c>
-      <c r="AT26" s="2" t="n">
+      <c r="AV26" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5180,56 +5392,64 @@
         </is>
       </c>
       <c r="AF27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG27" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AH27" s="2" t="inlineStr">
+      <c r="AG27" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [2, 0], [2, 1], [3, 0], [4, 0], [4, 1]]</t>
+        </is>
+      </c>
+      <c r="AH27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI27" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ27" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI27" s="2" t="n">
+      <c r="AK27" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ27" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK27" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL27" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM27" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN27" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO27" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP27" s="2" t="n">
+      <c r="AN27" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO27" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ27" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR27" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ27" s="2" t="n">
+      <c r="AS27" s="2" t="n">
         <v>55.5</v>
       </c>
-      <c r="AR27" s="2" t="n">
+      <c r="AT27" s="2" t="n">
         <v>60</v>
       </c>
-      <c r="AS27" s="2" t="inlineStr">
+      <c r="AU27" s="2" t="inlineStr">
         <is>
           <t>the knight, chess piece, L-shaped move</t>
         </is>
       </c>
-      <c r="AT27" s="2" t="n">
+      <c r="AV27" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5356,54 +5576,62 @@
         </is>
       </c>
       <c r="AF28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG28" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="AH28" s="2" t="inlineStr">
+      <c r="AG28" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 1], [2, 1], [3, 1], [4, 0], [4, 1]]</t>
+        </is>
+      </c>
+      <c r="AH28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI28" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AJ28" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI28" s="2" t="n">
+      <c r="AK28" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ28" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK28" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL28" s="2" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="AM28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN28" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN28" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AO28" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP28" s="2" t="n">
+      <c r="AP28" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ28" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR28" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ28" s="2" t="n">
+      <c r="AS28" s="2" t="n">
         <v>54.85714286</v>
       </c>
-      <c r="AR28" s="2" t="n">
+      <c r="AT28" s="2" t="n">
         <v>58</v>
       </c>
-      <c r="AS28" s="2" t="inlineStr">
+      <c r="AU28" s="2" t="inlineStr">
         <is>
           <t>the rook, chess piece, straight power</t>
         </is>
       </c>
-      <c r="AT28" s="2" t="n">
+      <c r="AV28" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5530,54 +5758,62 @@
         </is>
       </c>
       <c r="AF29" s="2" t="n">
+        <v>4</v>
+      </c>
+      <c r="AG29" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [1, 0], [1, 1], [2, 0]]</t>
+        </is>
+      </c>
+      <c r="AH29" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG29" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH29" s="2" t="inlineStr">
+      <c r="AI29" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ29" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI29" s="2" t="inlineStr"/>
-      <c r="AJ29" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL29" s="2" t="n">
-        <v>1</v>
+      <c r="AK29" s="2" t="inlineStr"/>
+      <c r="AL29" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM29" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN29" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AN29" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO29" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP29" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AP29" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR29" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS29" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="AR29" s="2" t="n">
+      <c r="AT29" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="AS29" s="2" t="inlineStr">
+      <c r="AU29" s="2" t="inlineStr">
         <is>
           <t>galaxy, spiral nebula, cosmic swirl</t>
         </is>
       </c>
-      <c r="AT29" s="2" t="n">
+      <c r="AV29" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5704,54 +5940,62 @@
         </is>
       </c>
       <c r="AF30" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG30" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 2], [1, 0], [1, 1], [1, 2], [2, 0], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH30" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG30" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH30" s="2" t="inlineStr">
+      <c r="AI30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ30" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI30" s="2" t="inlineStr"/>
-      <c r="AJ30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL30" s="2" t="n">
-        <v>1</v>
+      <c r="AK30" s="2" t="inlineStr"/>
+      <c r="AL30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM30" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN30" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AN30" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO30" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP30" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP30" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ30" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR30" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ30" s="2" t="n">
+      <c r="AS30" s="2" t="n">
         <v>43.33333333</v>
       </c>
-      <c r="AR30" s="2" t="n">
+      <c r="AT30" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="AS30" s="2" t="inlineStr">
+      <c r="AU30" s="2" t="inlineStr">
         <is>
           <t>lighthouse, beacon tower, guiding light</t>
         </is>
       </c>
-      <c r="AT30" s="2" t="n">
+      <c r="AV30" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -5878,54 +6122,62 @@
         </is>
       </c>
       <c r="AF31" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AG31" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [1, 2], [2, 0], [2, 1], [2, 2]]</t>
+        </is>
+      </c>
+      <c r="AH31" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG31" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH31" s="2" t="inlineStr">
+      <c r="AI31" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ31" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI31" s="2" t="inlineStr"/>
-      <c r="AJ31" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK31" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL31" s="2" t="n">
-        <v>2</v>
+      <c r="AK31" s="2" t="inlineStr"/>
+      <c r="AL31" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN31" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN31" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AO31" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP31" s="2" t="n">
+      <c r="AP31" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ31" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR31" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ31" s="2" t="n">
+      <c r="AS31" s="2" t="n">
         <v>41.5</v>
       </c>
-      <c r="AR31" s="2" t="n">
+      <c r="AT31" s="2" t="n">
         <v>45</v>
       </c>
-      <c r="AS31" s="2" t="inlineStr">
+      <c r="AU31" s="2" t="inlineStr">
         <is>
           <t>bastion, fortified tower, stronghold</t>
         </is>
       </c>
-      <c r="AT31" s="2" t="n">
+      <c r="AV31" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6054,56 +6306,64 @@
         </is>
       </c>
       <c r="AF32" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG32" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG32" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [2, 0]]</t>
+        </is>
+      </c>
+      <c r="AH32" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI32" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AH32" s="2" t="inlineStr">
+      <c r="AJ32" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI32" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AK32" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL32" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AL32" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN32" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN32" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO32" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP32" s="2" t="n">
-        <v>1</v>
+      <c r="AP32" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR32" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS32" s="2" t="n">
         <v>48.8</v>
       </c>
-      <c r="AR32" s="2" t="n">
+      <c r="AT32" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="AS32" s="2" t="inlineStr">
+      <c r="AU32" s="2" t="inlineStr">
         <is>
           <t>nebula, cosmic cloud, star nursery</t>
         </is>
       </c>
-      <c r="AT32" s="2" t="n">
+      <c r="AV32" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6234,56 +6494,64 @@
         </is>
       </c>
       <c r="AF33" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG33" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG33" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [0, 2], [0, 3], [1, 0], [1, 1], [2, 0]]</t>
+        </is>
+      </c>
+      <c r="AH33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI33" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AH33" s="2" t="inlineStr">
+      <c r="AJ33" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI33" s="2" t="n">
+      <c r="AK33" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ33" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK33" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL33" s="2" t="n">
-        <v>1</v>
+      <c r="AL33" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM33" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN33" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AN33" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO33" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP33" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP33" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ33" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR33" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ33" s="2" t="n">
+      <c r="AS33" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="AR33" s="2" t="n">
+      <c r="AT33" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="AS33" s="2" t="inlineStr">
+      <c r="AU33" s="2" t="inlineStr">
         <is>
           <t>quadrant, navigation instrument, star chart</t>
         </is>
       </c>
-      <c r="AT33" s="2" t="n">
+      <c r="AV33" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6410,54 +6678,62 @@
         </is>
       </c>
       <c r="AF34" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG34" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AG34" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 1], [0, 2], [0, 3], [1, 0], [1, 1], [1, 3], [2, 0]]</t>
+        </is>
+      </c>
+      <c r="AH34" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI34" s="2" t="n">
         <v>5</v>
       </c>
-      <c r="AH34" s="2" t="inlineStr">
+      <c r="AJ34" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI34" s="2" t="n">
+      <c r="AK34" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ34" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK34" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL34" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AM34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN34" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN34" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO34" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP34" s="2" t="n">
+      <c r="AP34" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ34" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR34" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ34" s="2" t="n">
+      <c r="AS34" s="2" t="n">
         <v>52</v>
       </c>
-      <c r="AR34" s="2" t="n">
+      <c r="AT34" s="2" t="n">
         <v>56</v>
       </c>
-      <c r="AS34" s="2" t="inlineStr">
+      <c r="AU34" s="2" t="inlineStr">
         <is>
           <t>comet path, orbital trail, stellar trajectory</t>
         </is>
       </c>
-      <c r="AT34" s="2" t="n">
+      <c r="AV34" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6584,56 +6860,64 @@
         </is>
       </c>
       <c r="AF35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG35" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AH35" s="2" t="inlineStr">
+      <c r="AG35" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [0, 2], [0, 3], [1, 0], [1, 3], [2, 0], [2, 3]]</t>
+        </is>
+      </c>
+      <c r="AH35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI35" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ35" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI35" s="2" t="n">
+      <c r="AK35" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AJ35" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL35" s="2" t="n">
-        <v>1</v>
+      <c r="AL35" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM35" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN35" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AN35" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO35" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP35" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
+      </c>
+      <c r="AP35" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR35" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS35" s="2" t="n">
         <v>58.5</v>
       </c>
-      <c r="AR35" s="2" t="n">
+      <c r="AT35" s="2" t="n">
         <v>63</v>
       </c>
-      <c r="AS35" s="2" t="inlineStr">
+      <c r="AU35" s="2" t="inlineStr">
         <is>
           <t>star harbor, celestial port, cosmic dock</t>
         </is>
       </c>
-      <c r="AT35" s="2" t="n">
+      <c r="AV35" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6760,54 +7044,62 @@
         </is>
       </c>
       <c r="AF36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG36" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AH36" s="2" t="inlineStr">
+      <c r="AG36" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 3], [1, 3], [2, 1], [2, 3], [3, 0], [3, 1], [3, 2], [3, 3]]</t>
+        </is>
+      </c>
+      <c r="AH36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI36" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ36" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI36" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ36" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AK36" s="2" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="AL36" s="2" t="n">
         <v>1</v>
       </c>
       <c r="AM36" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN36" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AN36" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO36" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP36" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP36" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ36" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR36" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ36" s="2" t="n">
+      <c r="AS36" s="2" t="n">
         <v>55.5</v>
       </c>
-      <c r="AR36" s="2" t="n">
+      <c r="AT36" s="2" t="n">
         <v>59</v>
       </c>
-      <c r="AS36" s="2" t="inlineStr">
+      <c r="AU36" s="2" t="inlineStr">
         <is>
           <t>space axis, cosmic alignment, stellar center</t>
         </is>
       </c>
-      <c r="AT36" s="2" t="n">
+      <c r="AV36" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -6934,56 +7226,64 @@
         </is>
       </c>
       <c r="AF37" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG37" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AH37" s="2" t="inlineStr">
+      <c r="AG37" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 3], [1, 3], [2, 2], [2, 3], [3, 0], [3, 1], [3, 2], [3, 3]]</t>
+        </is>
+      </c>
+      <c r="AH37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI37" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ37" s="2" t="inlineStr">
         <is>
           <t>streckad</t>
         </is>
       </c>
-      <c r="AI37" s="2" t="n">
+      <c r="AK37" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AJ37" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK37" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL37" s="2" t="n">
-        <v>2</v>
+      <c r="AL37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM37" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AN37" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+        <v>1</v>
+      </c>
+      <c r="AN37" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AO37" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP37" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AP37" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ37" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR37" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ37" s="2" t="n">
+      <c r="AS37" s="2" t="n">
         <v>59.5</v>
       </c>
-      <c r="AR37" s="2" t="n">
+      <c r="AT37" s="2" t="n">
         <v>64</v>
       </c>
-      <c r="AS37" s="2" t="inlineStr">
+      <c r="AU37" s="2" t="inlineStr">
         <is>
           <t>observatory, telescope dome, stargazing</t>
         </is>
       </c>
-      <c r="AT37" s="2" t="n">
+      <c r="AV37" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7118,54 +7418,62 @@
       <c r="AF38" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH38" s="2" t="inlineStr">
+      <c r="AG38" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0]]</t>
+        </is>
+      </c>
+      <c r="AH38" s="2" t="n">
+        <v>3</v>
+      </c>
+      <c r="AI38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ38" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI38" s="2" t="inlineStr"/>
-      <c r="AJ38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL38" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN38" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO38" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP38" s="2" t="n">
-        <v>1</v>
+      <c r="AK38" s="2" t="inlineStr"/>
+      <c r="AL38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN38" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP38" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR38" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS38" s="2" t="n">
         <v>45.33333333</v>
       </c>
-      <c r="AR38" s="2" t="n">
+      <c r="AT38" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS38" s="2" t="inlineStr">
+      <c r="AU38" s="2" t="inlineStr">
         <is>
           <t>harbor change, port transition, dock shift</t>
         </is>
       </c>
-      <c r="AT38" s="2" t="n">
+      <c r="AV38" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7294,56 +7602,64 @@
         </is>
       </c>
       <c r="AF39" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG39" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 1], [0, 2], [1, 0], [1, 1], [1, 2]]</t>
+        </is>
+      </c>
+      <c r="AH39" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG39" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH39" s="2" t="inlineStr">
+      <c r="AI39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ39" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI39" s="2" t="inlineStr"/>
-      <c r="AJ39" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK39" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL39" s="2" t="n">
-        <v>2</v>
+      <c r="AK39" s="2" t="inlineStr"/>
+      <c r="AL39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM39" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN39" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO39" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AP39" s="2" t="n">
+      <c r="AN39" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO39" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AP39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ39" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AR39" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ39" s="2" t="n">
+      <c r="AS39" s="2" t="n">
         <v>42.4</v>
       </c>
-      <c r="AR39" s="2" t="n">
+      <c r="AT39" s="2" t="n">
         <v>44</v>
       </c>
-      <c r="AS39" s="2" t="inlineStr">
+      <c r="AU39" s="2" t="inlineStr">
         <is>
           <t>birdsong, avian melody, morning chorus</t>
         </is>
       </c>
-      <c r="AT39" s="2" t="n">
+      <c r="AV39" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7472,58 +7788,66 @@
         </is>
       </c>
       <c r="AF40" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG40" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [2, 0], [2, 1]]</t>
+        </is>
+      </c>
+      <c r="AH40" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AG40" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH40" s="2" t="inlineStr">
+      <c r="AI40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ40" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI40" s="2" t="n">
+      <c r="AK40" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ40" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK40" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL40" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM40" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN40" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO40" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP40" s="2" t="n">
+      <c r="AL40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN40" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP40" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ40" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR40" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ40" s="2" t="n">
+      <c r="AS40" s="2" t="n">
         <v>47.33333333</v>
       </c>
-      <c r="AR40" s="2" t="n">
+      <c r="AT40" s="2" t="n">
         <v>50</v>
       </c>
-      <c r="AS40" s="2" t="inlineStr">
+      <c r="AU40" s="2" t="inlineStr">
         <is>
           <t>mountain slope, hillside, rocky incline</t>
         </is>
       </c>
-      <c r="AT40" s="2" t="n">
+      <c r="AV40" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7654,58 +7978,66 @@
         </is>
       </c>
       <c r="AF41" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AH41" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="AG41" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0]]</t>
+        </is>
+      </c>
+      <c r="AH41" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AJ41" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ41" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AK41" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AL41" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM41" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AN41" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AK41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AL41" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM41" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AN41" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AO41" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP41" s="2" t="n">
-        <v>1</v>
+      <c r="AP41" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR41" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS41" s="2" t="n">
         <v>48</v>
       </c>
-      <c r="AR41" s="2" t="n">
+      <c r="AT41" s="2" t="n">
         <v>47</v>
       </c>
-      <c r="AS41" s="2" t="inlineStr">
+      <c r="AU41" s="2" t="inlineStr">
         <is>
           <t>rose grove, flowering garden, romantic park</t>
         </is>
       </c>
-      <c r="AT41" s="2" t="n">
+      <c r="AV41" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -7832,58 +8164,66 @@
         </is>
       </c>
       <c r="AF42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG42" s="2" t="n">
+        <v>5</v>
+      </c>
+      <c r="AG42" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [0, 2], [1, 1], [1, 2]]</t>
+        </is>
+      </c>
+      <c r="AH42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI42" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AH42" s="2" t="inlineStr">
+      <c r="AJ42" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI42" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AK42" s="2" t="n">
         <v>2</v>
       </c>
-      <c r="AL42" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AM42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN42" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO42" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP42" s="2" t="n">
+      <c r="AL42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AM42" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AN42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP42" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ42" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR42" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ42" s="2" t="n">
+      <c r="AS42" s="2" t="n">
         <v>49.6</v>
       </c>
-      <c r="AR42" s="2" t="n">
+      <c r="AT42" s="2" t="n">
         <v>51</v>
       </c>
-      <c r="AS42" s="2" t="inlineStr">
+      <c r="AU42" s="2" t="inlineStr">
         <is>
           <t>leaf meadow, deciduous clearing, green pasture</t>
         </is>
       </c>
-      <c r="AT42" s="2" t="n">
+      <c r="AV42" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8010,56 +8350,64 @@
         </is>
       </c>
       <c r="AF43" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AG43" s="2" t="n">
+        <v>6</v>
+      </c>
+      <c r="AG43" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [1, 1], [2, 0], [3, 0]]</t>
+        </is>
+      </c>
+      <c r="AH43" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AI43" s="2" t="n">
         <v>4</v>
       </c>
-      <c r="AH43" s="2" t="inlineStr">
+      <c r="AJ43" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI43" s="2" t="n">
+      <c r="AK43" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ43" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK43" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL43" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AM43" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN43" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO43" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP43" s="2" t="n">
+      <c r="AM43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AO43" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP43" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ43" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR43" s="2" t="n">
         <v>0.9</v>
       </c>
-      <c r="AQ43" s="2" t="n">
+      <c r="AS43" s="2" t="n">
         <v>51.33333333</v>
       </c>
-      <c r="AR43" s="2" t="n">
+      <c r="AT43" s="2" t="n">
         <v>54</v>
       </c>
-      <c r="AS43" s="2" t="inlineStr">
+      <c r="AU43" s="2" t="inlineStr">
         <is>
           <t>mill hill, grinding slope, water mill</t>
         </is>
       </c>
-      <c r="AT43" s="2" t="n">
+      <c r="AV43" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8190,56 +8538,64 @@
         </is>
       </c>
       <c r="AF44" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG44" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AH44" s="2" t="inlineStr">
+        <v>3</v>
+      </c>
+      <c r="AG44" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 1]]</t>
+        </is>
+      </c>
+      <c r="AH44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI44" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AJ44" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI44" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AJ44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AK44" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AL44" s="2" t="n">
-        <v>1</v>
+      <c r="AL44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM44" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN44" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN44" s="2" t="n">
+        <v>1</v>
       </c>
       <c r="AO44" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP44" s="2" t="n">
-        <v>1</v>
+      <c r="AP44" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AQ44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR44" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AS44" s="2" t="n">
         <v>50.66666667</v>
       </c>
-      <c r="AR44" s="2" t="n">
+      <c r="AT44" s="2" t="n">
         <v>49</v>
       </c>
-      <c r="AS44" s="2" t="inlineStr">
+      <c r="AU44" s="2" t="inlineStr">
         <is>
           <t>river bank, stream edge, waterside</t>
         </is>
       </c>
-      <c r="AT44" s="2" t="n">
+      <c r="AV44" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8364,56 +8720,64 @@
         </is>
       </c>
       <c r="AF45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG45" s="2" t="n">
         <v>8</v>
       </c>
-      <c r="AH45" s="2" t="inlineStr">
+      <c r="AG45" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 0], [0, 1], [1, 0], [2, 0], [3, 0], [3, 1], [3, 2], [3, 3]]</t>
+        </is>
+      </c>
+      <c r="AH45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI45" s="2" t="n">
+        <v>8</v>
+      </c>
+      <c r="AJ45" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI45" s="2" t="n">
+      <c r="AK45" s="2" t="n">
         <v>3</v>
       </c>
-      <c r="AJ45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AK45" s="2" t="n">
-        <v>1</v>
-      </c>
       <c r="AL45" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AM45" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AN45" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="AO45" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AP45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AM45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AN45" s="2" t="n">
+        <v>2</v>
+      </c>
+      <c r="AO45" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AP45" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ45" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR45" s="2" t="n">
         <v>1.05</v>
       </c>
-      <c r="AQ45" s="2" t="n">
+      <c r="AS45" s="2" t="n">
         <v>56.5</v>
       </c>
-      <c r="AR45" s="2" t="n">
+      <c r="AT45" s="2" t="n">
         <v>61</v>
       </c>
-      <c r="AS45" s="2" t="inlineStr">
+      <c r="AU45" s="2" t="inlineStr">
         <is>
           <t>stone edge, rock ridge, granite brow</t>
         </is>
       </c>
-      <c r="AT45" s="2" t="n">
+      <c r="AV45" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -8542,56 +8906,64 @@
         </is>
       </c>
       <c r="AF46" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AG46" s="2" t="n">
         <v>7</v>
       </c>
-      <c r="AH46" s="2" t="inlineStr">
+      <c r="AG46" s="2" t="inlineStr">
+        <is>
+          <t>[[0, 3], [1, 1], [1, 3], [2, 0], [2, 1], [2, 2], [2, 3]]</t>
+        </is>
+      </c>
+      <c r="AH46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AI46" s="2" t="n">
+        <v>7</v>
+      </c>
+      <c r="AJ46" s="2" t="inlineStr">
         <is>
           <t>heldragen</t>
         </is>
       </c>
-      <c r="AI46" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="AJ46" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
-      </c>
       <c r="AK46" s="2" t="n">
-        <v>1</v>
-      </c>
-      <c r="AL46" s="2" t="n">
-        <v>2</v>
+        <v>2</v>
+      </c>
+      <c r="AL46" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
       </c>
       <c r="AM46" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AN46" s="2" t="inlineStr">
-        <is>
-          <t>-</t>
-        </is>
+      <c r="AN46" s="2" t="n">
+        <v>2</v>
       </c>
       <c r="AO46" s="2" t="n">
         <v>1</v>
       </c>
-      <c r="AP46" s="2" t="n">
+      <c r="AP46" s="2" t="inlineStr">
+        <is>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="AQ46" s="2" t="n">
+        <v>1</v>
+      </c>
+      <c r="AR46" s="2" t="n">
         <v>0.95</v>
       </c>
-      <c r="AQ46" s="2" t="n">
+      <c r="AS46" s="2" t="n">
         <v>53.71428571</v>
       </c>
-      <c r="AR46" s="2" t="n">
+      <c r="AT46" s="2" t="n">
         <v>57</v>
       </c>
-      <c r="AS46" s="2" t="inlineStr">
+      <c r="AU46" s="2" t="inlineStr">
         <is>
           <t>lake glimmer, water sparkle, shimmering shore</t>
         </is>
       </c>
-      <c r="AT46" s="2" t="n">
+      <c r="AV46" s="2" t="n">
         <v>1</v>
       </c>
     </row>
@@ -11918,7 +12290,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D47"/>
+  <dimension ref="A1:D49"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -12622,12 +12994,12 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>Förekomst</t>
+          <t>Antal rutor</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>Förekomst</t>
+          <t>F_rutor</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
@@ -12637,19 +13009,19 @@
       </c>
       <c r="D33" t="inlineStr">
         <is>
-          <t>Ej tryckt — speldata</t>
+          <t>Ej tryckt — brickans storlek; en ruta = 250 kvm (= BTA / 250)</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>Formfaktor</t>
+          <t>Form (rutor)</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>Formfaktor</t>
+          <t>F_form</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -12659,19 +13031,19 @@
       </c>
       <c r="D34" t="inlineStr">
         <is>
-          <t>Ej tryckt — styr brickans form (1–8)</t>
+          <t>Ej tryckt — brickans form som [rad, kolumn] per ruta (från brickorna)</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>Linjetyp</t>
+          <t>Förekomst</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>linjetyp</t>
+          <t>Förekomst</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -12681,19 +13053,19 @@
       </c>
       <c r="D35" t="inlineStr">
         <is>
-          <t>Ej tryckt — ramens linjestil</t>
+          <t>Ej tryckt — speldata</t>
         </is>
       </c>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>Antal krav</t>
+          <t>Formfaktor</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Antal krav</t>
+          <t>Formfaktor</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -12703,19 +13075,19 @@
       </c>
       <c r="D36" t="inlineStr">
         <is>
-          <t>Ej tryckt</t>
+          <t>Ej tryckt — styr brickans form (1–8)</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>Linjetyp</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>STA</t>
+          <t>linjetyp</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
@@ -12725,19 +13097,19 @@
       </c>
       <c r="D37" t="inlineStr">
         <is>
-          <t>Ej tryckt — kompetens</t>
+          <t>Ej tryckt — ramens linjestil</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>KOM</t>
+          <t>Antal krav</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>KOM</t>
+          <t>Antal krav</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
@@ -12747,19 +13119,19 @@
       </c>
       <c r="D38" t="inlineStr">
         <is>
-          <t>Ej tryckt — kompetens</t>
+          <t>Ej tryckt</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>SAM</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>SAM</t>
+          <t>STA</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -12776,12 +13148,12 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>NOG</t>
+          <t>KOM</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>NOG</t>
+          <t>KOM</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
@@ -12798,12 +13170,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>INN</t>
+          <t>SAM</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>INN</t>
+          <t>SAM</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -12820,12 +13192,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>ABM</t>
+          <t>NOG</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>ABM</t>
+          <t>NOG</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -12842,12 +13214,12 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>Skalfaktor</t>
+          <t>INN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>Skalfaktor</t>
+          <t>INN</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
@@ -12857,19 +13229,19 @@
       </c>
       <c r="D43" t="inlineStr">
         <is>
-          <t>Ej tryckt</t>
+          <t>Ej tryckt — kompetens</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>Intäkt/kvm nu</t>
+          <t>ABM</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>intäkt/kvm nu</t>
+          <t>ABM</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
@@ -12879,19 +13251,19 @@
       </c>
       <c r="D44" t="inlineStr">
         <is>
-          <t>Ej tryckt — beräkningsunderlag</t>
+          <t>Ej tryckt — kompetens</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>Förslag intäkt</t>
+          <t>Skalfaktor</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>förslag intäkt</t>
+          <t>Skalfaktor</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
@@ -12901,19 +13273,19 @@
       </c>
       <c r="D45" t="inlineStr">
         <is>
-          <t>Ej tryckt — beräkningsunderlag</t>
+          <t>Ej tryckt</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>Bildprompt (en)</t>
+          <t>Intäkt/kvm nu</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>namn_en</t>
+          <t>intäkt/kvm nu</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -12923,27 +13295,71 @@
       </c>
       <c r="D46" t="inlineStr">
         <is>
-          <t>Ej tryckt — underlag för bildgenerering</t>
+          <t>Ej tryckt — beräkningsunderlag</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
+          <t>Förslag intäkt</t>
+        </is>
+      </c>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>förslag intäkt</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
+          <t>Nej</t>
+        </is>
+      </c>
+      <c r="D47" t="inlineStr">
+        <is>
+          <t>Ej tryckt — beräkningsunderlag</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" t="inlineStr">
+        <is>
+          <t>Bildprompt (en)</t>
+        </is>
+      </c>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>namn_en</t>
+        </is>
+      </c>
+      <c r="C48" t="inlineStr">
+        <is>
+          <t>Nej</t>
+        </is>
+      </c>
+      <c r="D48" t="inlineStr">
+        <is>
+          <t>Ej tryckt — underlag för bildgenerering</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" t="inlineStr">
+        <is>
           <t>Antal exemplar</t>
         </is>
       </c>
-      <c r="B47" t="inlineStr">
+      <c r="B49" t="inlineStr">
         <is>
           <t>—</t>
         </is>
       </c>
-      <c r="C47" t="inlineStr">
+      <c r="C49" t="inlineStr">
         <is>
           <t>Nej</t>
         </is>
       </c>
-      <c r="D47" t="inlineStr">
+      <c r="D49" t="inlineStr">
         <is>
           <t>Antal tryckta kort (utskrift_config: 1)</t>
         </is>
@@ -12960,7 +13376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B13"/>
+  <dimension ref="A1:B15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13102,22 +13518,46 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Omtryck</t>
+          <t>Omtryck BTA</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr">
         <is>
-          <t>Marknadsvärde, energiklass, driftnetto (nu efter ränta, per år), räntekostnad och lån för förvaltningsbara typer kommer från data/forvaltning_2-1/F2-1_projektkort.csv — de tryckta värdena finns kvar i arv/ och i tryckfilens text.</t>
+          <t>Förskolan Regnbågen: BTA 2000 → 1750, så att kortet stämmer med brickans form (7 rutor).</t>
         </is>
       </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
+          <t>Former</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>Brickornas former från data/shapes.json; kontroll: rutor × 250 = BTA för alla 45.</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
+          <t>Omtryck</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>Marknadsvärde, energiklass, driftnetto (nu efter ränta, per år), räntekostnad och lån för förvaltningsbara typer kommer från data/forvaltning_2-1/F2-1_projektkort.csv — de tryckta värdena finns kvar i arv/ och i tryckfilens text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
           <t>Byggd med</t>
         </is>
       </c>
-      <c r="B13" s="2" t="inlineStr">
+      <c r="B15" s="2" t="inlineStr">
         <is>
           <t>verktyg/bygg_pu_projekt_excel.py</t>
         </is>

</xml_diff>

<commit_message>
Hyresrätter: anskaffningen sänkt cirka 5 % i omtrycket
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JCFLjpHxkTTwZndbAW5eBH
</commit_message>
<xml_diff>
--- a/kortdata/PU_projekt.xlsx
+++ b/kortdata/PU_projekt.xlsx
@@ -7318,7 +7318,7 @@
         <v>2</v>
       </c>
       <c r="H38" s="2" t="n">
-        <v>34</v>
+        <v>32</v>
       </c>
       <c r="I38" s="2" t="n">
         <v>1</v>
@@ -7508,7 +7508,7 @@
         <v>3</v>
       </c>
       <c r="H39" s="2" t="n">
-        <v>55</v>
+        <v>52</v>
       </c>
       <c r="I39" s="2" t="n">
         <v>1</v>
@@ -7694,7 +7694,7 @@
         <v>4</v>
       </c>
       <c r="H40" s="2" t="n">
-        <v>75</v>
+        <v>71</v>
       </c>
       <c r="I40" s="2" t="n">
         <v>1</v>
@@ -7882,7 +7882,7 @@
         <v>2</v>
       </c>
       <c r="H41" s="2" t="n">
-        <v>37</v>
+        <v>35</v>
       </c>
       <c r="I41" s="2" t="n">
         <v>1</v>
@@ -8072,7 +8072,7 @@
         <v>4</v>
       </c>
       <c r="H42" s="2" t="n">
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="I42" s="2" t="n">
         <v>1</v>
@@ -8258,7 +8258,7 @@
         <v>5</v>
       </c>
       <c r="H43" s="2" t="n">
-        <v>82</v>
+        <v>78</v>
       </c>
       <c r="I43" s="2" t="n">
         <v>1</v>
@@ -8300,7 +8300,7 @@
       </c>
       <c r="U43" s="2" t="inlineStr">
         <is>
-          <t>Balanserad</t>
+          <t>Kassako: billig att ta fram, stark i förvaltningen</t>
         </is>
       </c>
       <c r="V43" s="2" t="inlineStr"/>
@@ -8442,7 +8442,7 @@
         <v>2</v>
       </c>
       <c r="H44" s="2" t="n">
-        <v>39</v>
+        <v>37</v>
       </c>
       <c r="I44" s="2" t="n">
         <v>2</v>
@@ -8630,7 +8630,7 @@
         <v>7</v>
       </c>
       <c r="H45" s="2" t="n">
-        <v>122</v>
+        <v>116</v>
       </c>
       <c r="I45" s="2" t="n">
         <v>2</v>
@@ -8812,7 +8812,7 @@
         <v>6</v>
       </c>
       <c r="H46" s="2" t="n">
-        <v>101</v>
+        <v>96</v>
       </c>
       <c r="I46" s="2" t="n">
         <v>2</v>
@@ -8852,7 +8852,7 @@
       </c>
       <c r="U46" s="2" t="inlineStr">
         <is>
-          <t>Balanserad</t>
+          <t>Kassako: billig att ta fram, stark i förvaltningen</t>
         </is>
       </c>
       <c r="V46" s="2" t="inlineStr">
@@ -13376,7 +13376,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B15"/>
+  <dimension ref="A1:B16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="20" customWidth="1" min="1" max="1"/>
@@ -13530,34 +13530,46 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Former</t>
+          <t>Omtryck anskaffning</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr">
         <is>
-          <t>Brickornas former från data/shapes.json; kontroll: rutor × 250 = BTA för alla 45.</t>
+          <t>Hyresrätter: anskaffningen sänkt cirka 5 % (tryggt val ska kosta lite i Projektutvecklingen).</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Omtryck</t>
+          <t>Former</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr">
         <is>
-          <t>Marknadsvärde, energiklass, driftnetto (nu efter ränta, per år), räntekostnad och lån för förvaltningsbara typer kommer från data/forvaltning_2-1/F2-1_projektkort.csv — de tryckta värdena finns kvar i arv/ och i tryckfilens text.</t>
+          <t>Brickornas former från data/shapes.json; kontroll: rutor × 250 = BTA för alla 45.</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
+          <t>Omtryck</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>Marknadsvärde, energiklass, driftnetto (nu efter ränta, per år), räntekostnad och lån för förvaltningsbara typer kommer från data/forvaltning_2-1/F2-1_projektkort.csv — de tryckta värdena finns kvar i arv/ och i tryckfilens text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
           <t>Byggd med</t>
         </is>
       </c>
-      <c r="B15" s="2" t="inlineStr">
+      <c r="B16" s="2" t="inlineStr">
         <is>
           <t>verktyg/bygg_pu_projekt_excel.py</t>
         </is>

</xml_diff>